<commit_message>
Update car import logic and template for new Excel format
- Adjust import logic to match new Excel column structure: VIN, Car Name, License Plate, etc.
- Add support for reading and updating Car Name (TenXe).
- Update user instructions and template file to reflect new columns.
- Note: VIN length validation (17) differs from new doc (15).
</commit_message>
<xml_diff>
--- a/ChargePoint.CarManagement/wwwroot/template/DATA XE-TEMPLATE.xlsx
+++ b/ChargePoint.CarManagement/wwwroot/template/DATA XE-TEMPLATE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huytr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Estore\ChargePoint.CarManagement\ChargePoint.CarManagement\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D5DBBD-7585-4C52-B354-BE6C1E26150F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48DA0508-827B-4087-B6EE-5A27EA4B7B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{38A572B5-3AB4-49E8-81F2-D47B1E98768E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>STT</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>MÀU, LOẠI BIỂN</t>
+  </si>
+  <si>
+    <t>DÒNG XE</t>
   </si>
 </sst>
 </file>
@@ -115,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -124,6 +127,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3AED459-22D6-4FAF-8081-6B1CE9BC7913}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.7265625" bestFit="1" customWidth="1"/>
@@ -448,45 +456,50 @@
     <col min="5" max="5" width="9.26953125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.26953125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.26953125" style="6" customWidth="1"/>
     <col min="10" max="10" width="24" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.90625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F1048576" xr:uid="{4D100384-D3E6-4BFC-B21C-754B7CD45B27}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{4D100384-D3E6-4BFC-B21C-754B7CD45B27}">
       <formula1>"Trắng,Vàng"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>